<commit_message>
MADE MY FINAL CLUSTER ANALYSIS - HOPEFULLY
</commit_message>
<xml_diff>
--- a/analysis/data/raw_data/data_measurements_01.xlsx
+++ b/analysis/data/raw_data/data_measurements_01.xlsx
@@ -260,6 +260,9 @@
     <t xml:space="preserve">V36</t>
   </si>
   <si>
+    <t xml:space="preserve">d</t>
+  </si>
+  <si>
     <t xml:space="preserve">V37</t>
   </si>
   <si>
@@ -288,9 +291,6 @@
   </si>
   <si>
     <t xml:space="preserve">V45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d</t>
   </si>
   <si>
     <t xml:space="preserve">V46</t>
@@ -3108,7 +3108,7 @@
         <v>46</v>
       </c>
       <c r="F10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G10" t="s">
         <v>23</v>
@@ -3959,7 +3959,7 @@
         <v>46</v>
       </c>
       <c r="F25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G25" t="s">
         <v>61</v>
@@ -4644,7 +4644,7 @@
         <v>6</v>
       </c>
       <c r="G37" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H37" t="s">
         <v>38</v>
@@ -4687,7 +4687,7 @@
         <v>43</v>
       </c>
       <c r="C38" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D38" t="s">
         <v>57</v>
@@ -4744,7 +4744,7 @@
         <v>43</v>
       </c>
       <c r="C39" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D39" t="s">
         <v>57</v>
@@ -4801,7 +4801,7 @@
         <v>43</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D40" t="s">
         <v>57</v>
@@ -4858,7 +4858,7 @@
         <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D41" t="s">
         <v>57</v>
@@ -4915,7 +4915,7 @@
         <v>43</v>
       </c>
       <c r="C42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D42" t="s">
         <v>57</v>
@@ -4970,7 +4970,7 @@
         <v>43</v>
       </c>
       <c r="C43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D43" t="s">
         <v>57</v>
@@ -5025,7 +5025,7 @@
         <v>43</v>
       </c>
       <c r="C44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D44" t="s">
         <v>57</v>
@@ -5082,7 +5082,7 @@
         <v>43</v>
       </c>
       <c r="C45" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D45" t="s">
         <v>57</v>
@@ -5097,10 +5097,10 @@
         <v>29</v>
       </c>
       <c r="H45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J45" t="s">
         <v>36</v>
@@ -5139,7 +5139,7 @@
         <v>43</v>
       </c>
       <c r="C46" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D46" t="s">
         <v>57</v>
@@ -5151,7 +5151,7 @@
         <v>5</v>
       </c>
       <c r="G46" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H46" t="s">
         <v>38</v>
@@ -5538,7 +5538,7 @@
         <v>3</v>
       </c>
       <c r="G53" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H53" t="s">
         <v>103</v>
@@ -5595,7 +5595,7 @@
         <v>5</v>
       </c>
       <c r="G54" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H54" t="s">
         <v>71</v>
@@ -6391,7 +6391,7 @@
         <v>10</v>
       </c>
       <c r="G68" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H68" t="s">
         <v>71</v>
@@ -6560,13 +6560,13 @@
         <v>10</v>
       </c>
       <c r="G71" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H71" t="s">
         <v>71</v>
       </c>
       <c r="I71" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J71"/>
       <c r="K71"/>
@@ -7668,13 +7668,13 @@
         <v>5</v>
       </c>
       <c r="G91" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H91" t="s">
         <v>153</v>
       </c>
       <c r="I91" t="s">
-        <v>104</v>
+        <v>35</v>
       </c>
       <c r="J91"/>
       <c r="K91"/>
@@ -9283,7 +9283,7 @@
         <v>6</v>
       </c>
       <c r="G120" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H120" t="s">
         <v>54</v>
@@ -9457,10 +9457,10 @@
         <v>23</v>
       </c>
       <c r="H123" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="I123" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J123" t="s">
         <v>136</v>
@@ -10483,10 +10483,10 @@
         <v>23</v>
       </c>
       <c r="H141" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="I141" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J141" t="s">
         <v>36</v>
@@ -11346,10 +11346,10 @@
         <v>23</v>
       </c>
       <c r="H156" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="I156" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J156" t="s">
         <v>36</v>
@@ -11972,7 +11972,7 @@
         <v>71</v>
       </c>
       <c r="I167" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J167" t="s">
         <v>136</v>
@@ -12140,10 +12140,10 @@
         <v>23</v>
       </c>
       <c r="H170" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="I170" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J170" t="s">
         <v>136</v>
@@ -12194,7 +12194,7 @@
         <v>9</v>
       </c>
       <c r="G171" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H171" t="s">
         <v>103</v>
@@ -12308,7 +12308,7 @@
         <v>5</v>
       </c>
       <c r="G173" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H173" t="s">
         <v>24</v>
@@ -14199,7 +14199,7 @@
         <v>290</v>
       </c>
       <c r="I206" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="J206" t="s">
         <v>36</v>
@@ -14256,7 +14256,7 @@
         <v>290</v>
       </c>
       <c r="I207" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="J207" t="s">
         <v>36</v>
@@ -14313,7 +14313,7 @@
         <v>290</v>
       </c>
       <c r="I208" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="J208" t="s">
         <v>36</v>
@@ -14421,13 +14421,13 @@
         <v>5</v>
       </c>
       <c r="G210" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H210" t="s">
         <v>290</v>
       </c>
       <c r="I210" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="J210" t="s">
         <v>36</v>
@@ -14535,7 +14535,7 @@
         <v>9</v>
       </c>
       <c r="G212" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H212" t="s">
         <v>256</v>
@@ -15108,10 +15108,10 @@
         <v>29</v>
       </c>
       <c r="H222" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I222" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J222" t="s">
         <v>36</v>
@@ -15881,7 +15881,7 @@
         <v>5</v>
       </c>
       <c r="G236" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H236" t="s">
         <v>63</v>
@@ -15936,7 +15936,7 @@
         <v>5</v>
       </c>
       <c r="G237" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H237" t="s">
         <v>24</v>
@@ -15991,7 +15991,7 @@
         <v>5</v>
       </c>
       <c r="G238" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H238" t="s">
         <v>153</v>
@@ -16101,7 +16101,7 @@
         <v>5</v>
       </c>
       <c r="G240" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H240" t="s">
         <v>24</v>
@@ -16156,7 +16156,7 @@
         <v>5</v>
       </c>
       <c r="G241" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H241" t="s">
         <v>24</v>
@@ -16211,7 +16211,7 @@
         <v>5</v>
       </c>
       <c r="G242" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H242" t="s">
         <v>153</v>
@@ -16266,7 +16266,7 @@
         <v>5</v>
       </c>
       <c r="G243" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H243" t="s">
         <v>24</v>
@@ -16651,7 +16651,7 @@
         <v>5</v>
       </c>
       <c r="G250" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H250" t="s">
         <v>258</v>
@@ -16706,7 +16706,7 @@
         <v>5</v>
       </c>
       <c r="G251" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H251" t="s">
         <v>24</v>
@@ -16926,7 +16926,7 @@
         <v>5</v>
       </c>
       <c r="G255" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H255" t="s">
         <v>24</v>
@@ -16981,7 +16981,7 @@
         <v>5</v>
       </c>
       <c r="G256" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H256" t="s">
         <v>24</v>
@@ -17036,7 +17036,7 @@
         <v>5</v>
       </c>
       <c r="G257" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H257" t="s">
         <v>63</v>
@@ -17091,7 +17091,7 @@
         <v>5</v>
       </c>
       <c r="G258" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H258" t="s">
         <v>24</v>
@@ -17146,7 +17146,7 @@
         <v>5</v>
       </c>
       <c r="G259" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H259" t="s">
         <v>153</v>
@@ -19893,7 +19893,7 @@
         <v>46</v>
       </c>
       <c r="F309" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G309" t="s">
         <v>75</v>
@@ -19925,10 +19925,10 @@
         <v>66</v>
       </c>
       <c r="R309" t="n">
-        <v>160486.656</v>
+        <v>150456.24</v>
       </c>
       <c r="S309" t="n">
-        <v>160.486656</v>
+        <v>150.45624</v>
       </c>
     </row>
     <row r="310">
@@ -19948,7 +19948,7 @@
         <v>46</v>
       </c>
       <c r="F310" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G310" t="s">
         <v>29</v>
@@ -19980,10 +19980,10 @@
         <v>29.2</v>
       </c>
       <c r="R310" t="n">
-        <v>13386.448</v>
+        <v>13029.4760533333</v>
       </c>
       <c r="S310" t="n">
-        <v>13.386448</v>
+        <v>13.0294760533333</v>
       </c>
     </row>
     <row r="311">
@@ -22062,7 +22062,7 @@
         <v>71</v>
       </c>
       <c r="I347" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J347" t="s">
         <v>36</v>
@@ -22575,7 +22575,7 @@
         <v>464</v>
       </c>
       <c r="I356" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J356" t="s">
         <v>36</v>
@@ -22629,10 +22629,10 @@
         <v>23</v>
       </c>
       <c r="H357" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I357" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J357" t="s">
         <v>36</v>
@@ -22917,7 +22917,7 @@
         <v>464</v>
       </c>
       <c r="I362" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J362" t="s">
         <v>36</v>
@@ -22974,7 +22974,7 @@
         <v>464</v>
       </c>
       <c r="I363" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J363" t="s">
         <v>36</v>
@@ -23031,7 +23031,7 @@
         <v>464</v>
       </c>
       <c r="I364" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J364" t="s">
         <v>36</v>
@@ -23259,7 +23259,7 @@
         <v>290</v>
       </c>
       <c r="I368" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="J368" t="s">
         <v>36</v>
@@ -23316,7 +23316,7 @@
         <v>464</v>
       </c>
       <c r="I369" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J369" t="s">
         <v>36</v>
@@ -23601,7 +23601,7 @@
         <v>290</v>
       </c>
       <c r="I374" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="J374" t="s">
         <v>36</v>
@@ -24664,7 +24664,7 @@
         <v>3</v>
       </c>
       <c r="G393" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H393" t="s">
         <v>38</v>
@@ -25173,7 +25173,7 @@
         <v>290</v>
       </c>
       <c r="I402" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="J402"/>
       <c r="K402"/>
@@ -25393,7 +25393,7 @@
         <v>4</v>
       </c>
       <c r="G406" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H406" t="s">
         <v>34</v>
@@ -25450,7 +25450,7 @@
         <v>4</v>
       </c>
       <c r="G407" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H407" t="s">
         <v>34</v>
@@ -25511,7 +25511,7 @@
         <v>71</v>
       </c>
       <c r="I408" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J408" t="s">
         <v>136</v>
@@ -25629,7 +25629,7 @@
         <v>71</v>
       </c>
       <c r="I410" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J410"/>
       <c r="K410" t="s">
@@ -25846,16 +25846,16 @@
         <v>46</v>
       </c>
       <c r="F414" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G414" t="s">
         <v>29</v>
       </c>
       <c r="H414" t="s">
-        <v>24</v>
+        <v>242</v>
       </c>
       <c r="I414" t="s">
-        <v>25</v>
+        <v>242</v>
       </c>
       <c r="J414"/>
       <c r="K414" t="s">
@@ -25880,10 +25880,10 @@
         <v>30.8</v>
       </c>
       <c r="R414" t="n">
-        <v>15290.8119466667</v>
+        <v>7645.40597333333</v>
       </c>
       <c r="S414" t="n">
-        <v>15.2908119466667</v>
+        <v>7.64540597333333</v>
       </c>
     </row>
     <row r="415">
@@ -25903,16 +25903,16 @@
         <v>46</v>
       </c>
       <c r="F415" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G415" t="s">
         <v>29</v>
       </c>
       <c r="H415" t="s">
-        <v>24</v>
+        <v>242</v>
       </c>
       <c r="I415" t="s">
-        <v>25</v>
+        <v>242</v>
       </c>
       <c r="J415"/>
       <c r="K415" t="s">
@@ -25960,16 +25960,16 @@
         <v>46</v>
       </c>
       <c r="F416" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G416" t="s">
         <v>23</v>
       </c>
       <c r="H416" t="s">
-        <v>24</v>
+        <v>242</v>
       </c>
       <c r="I416" t="s">
-        <v>25</v>
+        <v>242</v>
       </c>
       <c r="J416" t="s">
         <v>36</v>
@@ -25996,10 +25996,10 @@
         <v>19.2</v>
       </c>
       <c r="R416" t="n">
-        <v>3704.09472</v>
+        <v>1852.04736</v>
       </c>
       <c r="S416" t="n">
-        <v>3.70409472</v>
+        <v>1.85204736</v>
       </c>
     </row>
     <row r="417">
@@ -30574,7 +30574,7 @@
         <v>71</v>
       </c>
       <c r="I503" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J503"/>
       <c r="K503"/>
@@ -33014,10 +33014,10 @@
         <v>29</v>
       </c>
       <c r="H546" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I546" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J546"/>
       <c r="K546"/>
@@ -33636,7 +33636,7 @@
         <v>71</v>
       </c>
       <c r="I557" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="J557" t="s">
         <v>136</v>
@@ -35012,10 +35012,10 @@
       </c>
       <c r="G584"/>
       <c r="H584" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I584" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J584"/>
       <c r="K584"/>
@@ -35062,7 +35062,7 @@
         <v>71</v>
       </c>
       <c r="I585" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="J585"/>
       <c r="K585"/>
@@ -35192,7 +35192,7 @@
         <v>22</v>
       </c>
       <c r="F588" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G588"/>
       <c r="H588"/>
@@ -36158,7 +36158,7 @@
         <v>5</v>
       </c>
       <c r="G609" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H609" t="s">
         <v>38</v>
@@ -36323,7 +36323,7 @@
         <v>4</v>
       </c>
       <c r="G612" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H612" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
Included a count of type, size, rim, base per site dependent on time. I made minor changes in the 10_timelinedata spreadsheet
</commit_message>
<xml_diff>
--- a/analysis/data/raw_data/data_measurements_01.xlsx
+++ b/analysis/data/raw_data/data_measurements_01.xlsx
@@ -14190,7 +14190,7 @@
         <v>46</v>
       </c>
       <c r="F206" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G206" t="s">
         <v>29</v>
@@ -14418,7 +14418,7 @@
         <v>46</v>
       </c>
       <c r="F210" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G210" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Removed the cluster analysis visualisations to the gibberish folder. Downloaded the new cluster analysis and descriptive statistics spreadsheets based on 11_timelinedata
</commit_message>
<xml_diff>
--- a/analysis/data/raw_data/data_measurements_01.xlsx
+++ b/analysis/data/raw_data/data_measurements_01.xlsx
@@ -14190,7 +14190,7 @@
         <v>46</v>
       </c>
       <c r="F206" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G206" t="s">
         <v>29</v>
@@ -14418,7 +14418,7 @@
         <v>46</v>
       </c>
       <c r="F210" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G210" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
New dataset 12_timelinedata with new type numbers (12 lids is deleted). Just small changes in the code
</commit_message>
<xml_diff>
--- a/analysis/data/raw_data/data_measurements_01.xlsx
+++ b/analysis/data/raw_data/data_measurements_01.xlsx
@@ -5374,7 +5374,7 @@
         <v>46</v>
       </c>
       <c r="F50" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G50"/>
       <c r="H50" t="s">
@@ -7227,7 +7227,7 @@
         <v>46</v>
       </c>
       <c r="F83" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G83"/>
       <c r="H83" t="s">
@@ -20174,7 +20174,7 @@
         <v>46</v>
       </c>
       <c r="F314" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G314"/>
       <c r="H314" t="s">
@@ -27326,7 +27326,7 @@
         <v>46</v>
       </c>
       <c r="F440" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G440"/>
       <c r="H440" t="s">
@@ -27377,7 +27377,7 @@
         <v>46</v>
       </c>
       <c r="F441" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G441"/>
       <c r="H441" t="s">
@@ -27428,7 +27428,7 @@
         <v>46</v>
       </c>
       <c r="F442" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G442"/>
       <c r="H442" t="s">
@@ -27479,7 +27479,7 @@
         <v>46</v>
       </c>
       <c r="F443" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G443"/>
       <c r="H443" t="s">
@@ -27530,7 +27530,7 @@
         <v>46</v>
       </c>
       <c r="F444" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G444"/>
       <c r="H444" t="s">
@@ -27581,7 +27581,7 @@
         <v>46</v>
       </c>
       <c r="F445" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G445"/>
       <c r="H445" t="s">
@@ -27632,7 +27632,7 @@
         <v>46</v>
       </c>
       <c r="F446" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G446"/>
       <c r="H446" t="s">
@@ -27683,7 +27683,7 @@
         <v>46</v>
       </c>
       <c r="F447" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G447"/>
       <c r="H447" t="s">
@@ -27734,7 +27734,7 @@
         <v>46</v>
       </c>
       <c r="F448" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G448"/>
       <c r="H448" t="s">
@@ -27785,7 +27785,7 @@
         <v>46</v>
       </c>
       <c r="F449" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G449"/>
       <c r="H449" t="s">
@@ -27836,7 +27836,7 @@
         <v>46</v>
       </c>
       <c r="F450" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G450"/>
       <c r="H450" t="s">
@@ -27887,7 +27887,7 @@
         <v>46</v>
       </c>
       <c r="F451" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G451"/>
       <c r="H451" t="s">
@@ -27936,7 +27936,7 @@
         <v>46</v>
       </c>
       <c r="F452" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G452"/>
       <c r="H452" t="s">
@@ -27985,7 +27985,7 @@
         <v>46</v>
       </c>
       <c r="F453" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G453"/>
       <c r="H453" t="s">
@@ -28034,7 +28034,7 @@
         <v>46</v>
       </c>
       <c r="F454" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G454"/>
       <c r="H454" t="s">
@@ -28083,7 +28083,7 @@
         <v>46</v>
       </c>
       <c r="F455" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G455"/>
       <c r="H455" t="s">
@@ -28132,7 +28132,7 @@
         <v>46</v>
       </c>
       <c r="F456" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G456"/>
       <c r="H456" t="s">
@@ -28181,7 +28181,7 @@
         <v>46</v>
       </c>
       <c r="F457" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G457"/>
       <c r="H457" t="s">
@@ -28230,7 +28230,7 @@
         <v>46</v>
       </c>
       <c r="F458" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G458"/>
       <c r="H458" t="s">
@@ -28279,7 +28279,7 @@
         <v>46</v>
       </c>
       <c r="F459" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G459"/>
       <c r="H459" t="s">
@@ -28328,7 +28328,7 @@
         <v>46</v>
       </c>
       <c r="F460" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G460"/>
       <c r="H460" t="s">
@@ -28377,7 +28377,7 @@
         <v>46</v>
       </c>
       <c r="F461" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G461"/>
       <c r="H461" t="s">
@@ -28426,7 +28426,7 @@
         <v>46</v>
       </c>
       <c r="F462" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G462"/>
       <c r="H462" t="s">
@@ -28475,7 +28475,7 @@
         <v>46</v>
       </c>
       <c r="F463" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G463"/>
       <c r="H463" t="s">
@@ -28524,7 +28524,7 @@
         <v>46</v>
       </c>
       <c r="F464" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G464"/>
       <c r="H464" t="s">
@@ -28573,7 +28573,7 @@
         <v>46</v>
       </c>
       <c r="F465" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G465"/>
       <c r="H465" t="s">
@@ -28622,7 +28622,7 @@
         <v>46</v>
       </c>
       <c r="F466" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G466"/>
       <c r="H466" t="s">
@@ -28671,7 +28671,7 @@
         <v>46</v>
       </c>
       <c r="F467" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G467"/>
       <c r="H467" t="s">
@@ -28720,7 +28720,7 @@
         <v>46</v>
       </c>
       <c r="F468" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G468"/>
       <c r="H468" t="s">
@@ -28769,7 +28769,7 @@
         <v>46</v>
       </c>
       <c r="F469" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G469"/>
       <c r="H469" t="s">
@@ -28820,7 +28820,7 @@
         <v>46</v>
       </c>
       <c r="F470" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G470"/>
       <c r="H470" t="s">
@@ -29148,7 +29148,7 @@
         <v>46</v>
       </c>
       <c r="F476" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G476"/>
       <c r="H476" t="s">
@@ -29201,7 +29201,7 @@
         <v>46</v>
       </c>
       <c r="F477" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G477"/>
       <c r="H477" t="s">
@@ -29254,7 +29254,7 @@
         <v>46</v>
       </c>
       <c r="F478" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G478"/>
       <c r="H478" t="s">
@@ -29702,7 +29702,7 @@
         <v>46</v>
       </c>
       <c r="F486" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G486"/>
       <c r="H486" t="s">
@@ -29753,7 +29753,7 @@
         <v>46</v>
       </c>
       <c r="F487" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G487"/>
       <c r="H487" t="s">
@@ -29804,7 +29804,7 @@
         <v>46</v>
       </c>
       <c r="F488" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G488"/>
       <c r="H488" t="s">
@@ -29857,7 +29857,7 @@
         <v>46</v>
       </c>
       <c r="F489" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G489"/>
       <c r="H489" t="s">
@@ -29906,7 +29906,7 @@
         <v>46</v>
       </c>
       <c r="F490" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G490"/>
       <c r="H490" t="s">
@@ -29957,7 +29957,7 @@
         <v>46</v>
       </c>
       <c r="F491" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G491"/>
       <c r="H491" t="s">
@@ -30008,7 +30008,7 @@
         <v>46</v>
       </c>
       <c r="F492" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G492"/>
       <c r="H492" t="s">
@@ -30059,7 +30059,7 @@
         <v>46</v>
       </c>
       <c r="F493" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G493"/>
       <c r="H493" t="s">
@@ -30110,7 +30110,7 @@
         <v>46</v>
       </c>
       <c r="F494" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G494"/>
       <c r="H494" t="s">
@@ -30161,7 +30161,7 @@
         <v>46</v>
       </c>
       <c r="F495" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G495"/>
       <c r="H495" t="s">
@@ -30212,7 +30212,7 @@
         <v>46</v>
       </c>
       <c r="F496" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G496"/>
       <c r="H496" t="s">
@@ -30263,7 +30263,7 @@
         <v>46</v>
       </c>
       <c r="F497" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G497"/>
       <c r="H497" t="s">
@@ -30314,7 +30314,7 @@
         <v>46</v>
       </c>
       <c r="F498" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G498"/>
       <c r="H498" t="s">
@@ -30365,7 +30365,7 @@
         <v>46</v>
       </c>
       <c r="F499" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G499"/>
       <c r="H499" t="s">
@@ -30416,7 +30416,7 @@
         <v>46</v>
       </c>
       <c r="F500" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G500"/>
       <c r="H500" t="s">
@@ -30465,7 +30465,7 @@
         <v>46</v>
       </c>
       <c r="F501" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G501"/>
       <c r="H501" t="s">
@@ -30516,7 +30516,7 @@
         <v>46</v>
       </c>
       <c r="F502" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G502"/>
       <c r="H502" t="s">
@@ -33973,7 +33973,7 @@
         <v>46</v>
       </c>
       <c r="F563" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G563"/>
       <c r="H563" t="s">
@@ -34138,7 +34138,7 @@
         <v>46</v>
       </c>
       <c r="F566" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G566"/>
       <c r="H566" t="s">

</xml_diff>